<commit_message>
Phase 2: Completing phase
</commit_message>
<xml_diff>
--- a/reports/phase2_tables_appendix_v1.xlsx
+++ b/reports/phase2_tables_appendix_v1.xlsx
@@ -4102,7 +4102,7 @@
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="39" customWidth="1" min="5" max="5"/>
     <col width="47" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="43" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>میانه‌ی وام وام‌گیران خوشه (میلیون تومان)</t>
+          <t>میانه‌ی مبلغ وام در خوشه (میلیون تومان)</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">

</xml_diff>